<commit_message>
feat: implement dynamic partners and reports settings CRUD, split period to year/month, add columns to orgunits Excel mapping
</commit_message>
<xml_diff>
--- a/config/mappings/pathfinder.xlsx
+++ b/config/mappings/pathfinder.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,6 +563,21 @@
           <t>Destination UID</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -575,6 +590,9 @@
           <t>DEST_OU_x1WE</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -587,6 +605,9 @@
           <t>DEST_OU_001</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -599,6 +620,9 @@
           <t>DEST_OU_002</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>